<commit_message>
v1 ready (no ui)
</commit_message>
<xml_diff>
--- a/exports/contentsquare_kpis.xlsx
+++ b/exports/contentsquare_kpis.xlsx
@@ -27,12 +27,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +65,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,27 +456,27 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>metric_value</t>
+          <t>metric_currency</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>metric_start_date</t>
+          <t>metric_extra_json</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>metric_end_date</t>
+          <t>metric_value_segment_6383684</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>metric_currency</t>
+          <t>metric_value_segment_6383688</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>metric_extra_json</t>
+          <t>metric_value_segment_6383692</t>
         </is>
       </c>
     </row>
@@ -475,28 +496,24 @@
           <t>bounceRate</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>33.34855182116247</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2.715695801155833</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>2.465055346562023</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>2.544121574053844</v>
       </c>
     </row>
     <row r="3">
@@ -515,28 +532,24 @@
           <t>cartAverage</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>30.29979577341555</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>30.40657149205644</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>30.33709745762712</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>30.04109806105402</v>
       </c>
     </row>
     <row r="4">
@@ -555,28 +568,24 @@
           <t>pageviewAverage</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>5.14131240459546</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>20.62541553725771</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>21.36038364001298</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>21.4331075668196</v>
       </c>
     </row>
     <row r="5">
@@ -595,28 +604,24 @@
           <t>revenueSum</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>2943534</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>547379</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>601402</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>593401</v>
       </c>
     </row>
     <row r="6">
@@ -635,28 +640,24 @@
           <t>sessionTimeAverage</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>232.3897834294591</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>697.7018992993402</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>689.0745506412028</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>691.8799663049547</v>
       </c>
     </row>
     <row r="7">
@@ -675,28 +676,24 @@
           <t>conversionCount</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>91554</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>16988</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>18721</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>18638</v>
       </c>
     </row>
     <row r="8">
@@ -715,28 +712,24 @@
           <t>conversionRate</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>1.840572568967191</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>21.72045210453639</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>22.50039061091547</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>22.62277571432039</v>
       </c>
     </row>
     <row r="9">
@@ -755,28 +748,24 @@
           <t>visits</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4974213</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:10.544Z</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>78212</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>83203</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>82386</v>
       </c>
     </row>
   </sheetData>
@@ -841,27 +830,27 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>metric_value</t>
+          <t>metric_currency</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>metric_start_date</t>
+          <t>metric_extra_json</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>metric_end_date</t>
+          <t>metric_value_segment_6383684</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>metric_currency</t>
+          <t>metric_value_segment_6383688</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>metric_extra_json</t>
+          <t>metric_value_segment_6383692</t>
         </is>
       </c>
     </row>
@@ -902,28 +891,24 @@
           <t>activityRate</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>25.9353951833841</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>26.76498567101016</v>
+      </c>
+      <c r="M2" s="1" t="n">
+        <v>24.22047136119623</v>
+      </c>
+      <c r="N2" s="1" t="n">
+        <v>24.28297499282402</v>
       </c>
     </row>
     <row r="3">
@@ -963,28 +948,24 @@
           <t>bounceRate</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>15.93358063946299</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>4.957805907172996</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>4.991087344028521</v>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>4.718875502008032</v>
       </c>
     </row>
     <row r="4">
@@ -1024,28 +1005,24 @@
           <t>elapsedTime</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>15.02682832148374</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>15.29983147002454</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>14.18640837017347</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>14.41020172933755</v>
       </c>
     </row>
     <row r="5">
@@ -1085,28 +1062,24 @@
           <t>exitRate</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>2.305428792299444</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>2.178627263099501</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>2.238763199747826</v>
+      </c>
+      <c r="N5" s="1" t="n">
+        <v>2.170508758512692</v>
       </c>
     </row>
     <row r="6">
@@ -1146,28 +1119,24 @@
           <t>foldHeight</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>743.3385461727564</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>745.7071755853545</v>
+      </c>
+      <c r="M6" s="1" t="n">
+        <v>738.2385019381372</v>
+      </c>
+      <c r="N6" s="1" t="n">
+        <v>737.8796066290294</v>
       </c>
     </row>
     <row r="7">
@@ -1207,28 +1176,24 @@
           <t>interactionTime</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>5.341031447357038</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>5.455715566930254</v>
+      </c>
+      <c r="M7" s="1" t="n">
+        <v>5.023319826184578</v>
+      </c>
+      <c r="N7" s="1" t="n">
+        <v>5.053522982364993</v>
       </c>
     </row>
     <row r="8">
@@ -1268,28 +1233,24 @@
           <t>landingRate</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>0.1138068106772138</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1.212090216335089</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>1.348509068182638</v>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>1.208957941372823</v>
       </c>
     </row>
     <row r="9">
@@ -1329,28 +1290,24 @@
           <t>loadingTime</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>0.8323254266474804</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0.8209079861111112</v>
+      </c>
+      <c r="M9" s="1" t="n">
+        <v>0.8185043390797876</v>
+      </c>
+      <c r="N9" s="1" t="n">
+        <v>0.8201291988845227</v>
       </c>
     </row>
     <row r="10">
@@ -1390,28 +1347,24 @@
           <t>pageHeight</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>1627.156737051445</v>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1657.429093751576</v>
+      </c>
+      <c r="M10" s="1" t="n">
+        <v>1570.228382502543</v>
+      </c>
+      <c r="N10" s="1" t="n">
+        <v>1574.205914272188</v>
       </c>
     </row>
     <row r="11">
@@ -1451,28 +1404,24 @@
           <t>scrollRate</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>65.52332123992694</v>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>67.72717709355469</v>
+      </c>
+      <c r="M11" s="1" t="n">
+        <v>62.81695170647178</v>
+      </c>
+      <c r="N11" s="1" t="n">
+        <v>62.62669978077236</v>
       </c>
     </row>
     <row r="12">
@@ -1512,28 +1461,24 @@
           <t>conversionRate</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>59.14016513124726</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>60.346116867856</v>
+      </c>
+      <c r="M12" s="1" t="n">
+        <v>58.23254364089775</v>
+      </c>
+      <c r="N12" s="1" t="n">
+        <v>58.70251167487063</v>
       </c>
     </row>
     <row r="13">
@@ -1573,28 +1518,24 @@
           <t>uniqueVisits</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>130451</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>24573</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>28047</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>27890</v>
       </c>
     </row>
     <row r="14">
@@ -1634,28 +1575,24 @@
           <t>views</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>641616</v>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>118974</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>139586</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>137295</v>
       </c>
     </row>
     <row r="15">
@@ -1695,28 +1632,24 @@
           <t>viewsVisits</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>4.201064644758294</v>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>4.236513193034932</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>4.351184538653366</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>4.332165846270352</v>
       </c>
     </row>
     <row r="16">
@@ -1756,28 +1689,24 @@
           <t>visits</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>152727</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.078Z</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>28083</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>32080</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>31692</v>
       </c>
     </row>
     <row r="17">
@@ -1817,23 +1746,19 @@
           <t>largestContentfulPaint</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>2.92</v>
-      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.187Z</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
           <t>{"metricType": "Quantile", "quantile": 0.75}</t>
         </is>
+      </c>
+      <c r="L17" t="n">
+        <v>2.926</v>
+      </c>
+      <c r="M17" s="1" t="n">
+        <v>2.842</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>2.956</v>
       </c>
     </row>
     <row r="18">
@@ -1873,23 +1798,19 @@
           <t>cumulativeLayoutShift</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>0.712883</v>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.187Z</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
           <t>{"metricType": "Quantile", "quantile": 0.75}</t>
         </is>
+      </c>
+      <c r="L18" t="n">
+        <v>0.8196560000000001</v>
+      </c>
+      <c r="M18" s="1" t="n">
+        <v>0.427963</v>
+      </c>
+      <c r="N18" s="1" t="n">
+        <v>0.430092</v>
       </c>
     </row>
     <row r="19">
@@ -1929,23 +1850,19 @@
           <t>interactionToNextPaint</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>{"metricType": "Quantile", "quantile": 0.75}</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="M19" s="1" t="n">
         <v>0.16</v>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.187Z</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>{"metricType": "Quantile", "quantile": 0.75}</t>
-        </is>
+      <c r="N19" s="1" t="n">
+        <v>0.16</v>
       </c>
     </row>
     <row r="20">
@@ -1985,23 +1902,19 @@
           <t>firstInputDelay</t>
         </is>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>{"metricType": "Quantile", "quantile": 0.75}</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
         <v>0</v>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.187Z</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>{"metricType": "Quantile", "quantile": 0.75}</t>
-        </is>
+      <c r="M20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -2041,23 +1954,19 @@
           <t>firstContentfulPaint</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>0.738</v>
-      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.187Z</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
           <t>{"metricType": "Quantile", "quantile": 0.75}</t>
         </is>
+      </c>
+      <c r="L21" t="n">
+        <v>0.744</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>0.74</v>
       </c>
     </row>
     <row r="22">
@@ -2097,23 +2006,19 @@
           <t>timeToFirstByte</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>0.448</v>
-      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.187Z</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
           <t>{"metricType": "Quantile", "quantile": 0.75}</t>
         </is>
+      </c>
+      <c r="L22" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="M22" s="1" t="n">
+        <v>0.431</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0.442</v>
       </c>
     </row>
     <row r="23">
@@ -2156,28 +2061,24 @@
           <t>conversionRate</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>77.61107074357011</v>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-01-31T00:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2026-03-02T11:12:12.317Z</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>78.51725243029591</v>
+      </c>
+      <c r="M23" s="1" t="n">
+        <v>77.27867830423941</v>
+      </c>
+      <c r="N23" s="1" t="n">
+        <v>77.82721191467878</v>
       </c>
     </row>
   </sheetData>

</xml_diff>